<commit_message>
Updated the system identification portion of the documentation.
</commit_message>
<xml_diff>
--- a/documentation/book/src/attachments/channel_table_template.xlsx
+++ b/documentation/book/src/attachments/channel_table_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dprohe\Documents\Local_Repositories\Rattlesnake_Overhaul\documentation\report\attachments\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dprohe\Documents\Local_Repositories\Rattlesnake_External\documentation\book\src\attachments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB9D9DF5-5F0C-43F5-A323-5391862C8BFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FF3AC93-7765-4E91-AF2F-E97635A6914D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Channel Table" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="26">
   <si>
     <t>Test Article Definition</t>
   </si>
@@ -98,15 +98,6 @@
   </si>
   <si>
     <t>Abort Level (EU)</t>
-  </si>
-  <si>
-    <t>Environment Table</t>
-  </si>
-  <si>
-    <t>Environment 1 Name</t>
-  </si>
-  <si>
-    <t>Environment 2 Name</t>
   </si>
 </sst>
 </file>
@@ -447,7 +438,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y502"/>
+  <dimension ref="A1:W502"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
@@ -477,7 +468,7 @@
     <col min="26" max="26" width="6.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -510,11 +501,8 @@
         <v>4</v>
       </c>
       <c r="W1" s="1"/>
-      <c r="X1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="2" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -584,79 +572,73 @@
       <c r="W2" t="s">
         <v>25</v>
       </c>
-      <c r="X2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>14</v>
       </c>

</xml_diff>